<commit_message>
feat(roster): auto-generate roll numbers on import and remove roll number from sample template
</commit_message>
<xml_diff>
--- a/public/templates/nexora-student-roster.xlsx
+++ b/public/templates/nexora-student-roster.xlsx
@@ -259,60 +259,49 @@
     <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>Roll number</x:v>
+        <x:v>First name</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str">
-        <x:v>First name</x:v>
+        <x:v>Father's name</x:v>
       </x:c>
       <x:c r="C1" s="2" t="str">
-        <x:v>Father's name</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="str">
         <x:v>Grandfather's name</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" t="str">
-        <x:v>1</x:v>
+        <x:v>Hana</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Hana</x:v>
+        <x:v>Dawit</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Dawit</x:v>
-      </x:c>
-      <x:c r="D2" t="str">
         <x:v>Getachew</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" t="str"/>
+      <x:c r="A3" t="str">
+        <x:v>Samuel</x:v>
+      </x:c>
       <x:c r="B3" t="str">
-        <x:v>Samuel</x:v>
+        <x:v>Abebe</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Abebe</x:v>
-      </x:c>
-      <x:c r="D3" t="str">
         <x:v>Tesfaye</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" t="str">
-        <x:v>3</x:v>
+        <x:v>Mekdes</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Mekdes</x:v>
+        <x:v>Kebede</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Kebede</x:v>
-      </x:c>
-      <x:c r="D4" t="str">
         <x:v>Tadesse</x:v>
       </x:c>
     </x:row>

</xml_diff>